<commit_message>
Update inventario_expandido.xlsx - 09/10/2026
</commit_message>
<xml_diff>
--- a/inventario_expandido.xlsx
+++ b/inventario_expandido.xlsx
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="J5" s="2" t="n">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="K5" s="2" t="n">
         <v>427</v>
@@ -791,7 +791,7 @@
         <v>391</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>1118</v>
+        <v>1116</v>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
@@ -898,10 +898,10 @@
         <v>92</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
@@ -1115,13 +1115,13 @@
         <v>28</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L11" s="2" t="n">
         <v>154</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="N11" s="4" t="inlineStr">
         <is>
@@ -1170,13 +1170,13 @@
         <v>10</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="L12" s="2" t="n">
         <v>13</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="N12" s="4" t="inlineStr">
         <is>
@@ -1489,7 +1489,7 @@
         </is>
       </c>
       <c r="J18" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="K18" s="2" t="n">
         <v>0</v>
@@ -1498,7 +1498,7 @@
         <v>0</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
@@ -2078,10 +2078,10 @@
         <v>7</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="N29" s="6" t="inlineStr">
         <is>
@@ -2455,7 +2455,7 @@
         </is>
       </c>
       <c r="J36" s="2" t="n">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="K36" s="2" t="n">
         <v>12</v>
@@ -2464,7 +2464,7 @@
         <v>185</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
@@ -2565,7 +2565,7 @@
         </is>
       </c>
       <c r="J38" s="2" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="K38" s="2" t="n">
         <v>239</v>
@@ -2574,7 +2574,7 @@
         <v>119</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
@@ -2675,7 +2675,7 @@
         </is>
       </c>
       <c r="J40" s="2" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="K40" s="2" t="n">
         <v>607</v>
@@ -2684,7 +2684,7 @@
         <v>174</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>844</v>
+        <v>838</v>
       </c>
       <c r="N40" s="4" t="inlineStr">
         <is>
@@ -2733,13 +2733,13 @@
         <v>99</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="L41" s="2" t="n">
         <v>18</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="N41" s="4" t="inlineStr">
         <is>
@@ -2788,13 +2788,13 @@
         <v>142</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>86</v>
       </c>
       <c r="M42" s="2" t="n">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
@@ -2846,10 +2846,10 @@
         <v>52</v>
       </c>
       <c r="L43" s="2" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M43" s="2" t="n">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="N43" s="4" t="inlineStr">
         <is>
@@ -2895,7 +2895,7 @@
         </is>
       </c>
       <c r="J44" s="2" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="K44" s="2" t="n">
         <v>198</v>
@@ -2904,11 +2904,11 @@
         <v>39</v>
       </c>
       <c r="M44" s="2" t="n">
-        <v>247</v>
-      </c>
-      <c r="N44" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>244</v>
+      </c>
+      <c r="N44" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O44" s="2" t="n">
@@ -3173,13 +3173,13 @@
         <v>21</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="L49" s="2" t="n">
         <v>62</v>
       </c>
       <c r="M49" s="2" t="n">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="N49" s="4" t="inlineStr">
         <is>
@@ -3338,13 +3338,13 @@
         <v>2</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="L52" s="2" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="N52" s="6" t="inlineStr">
         <is>
@@ -4823,13 +4823,13 @@
         <v>87</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="L79" s="2" t="n">
         <v>170</v>
       </c>
       <c r="M79" s="2" t="n">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="N79" s="4" t="inlineStr">
         <is>
@@ -7776,13 +7776,13 @@
         <v>20</v>
       </c>
       <c r="K132" s="2" t="n">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="L132" s="2" t="n">
         <v>149</v>
       </c>
       <c r="M132" s="2" t="n">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="N132" s="4" t="inlineStr">
         <is>
@@ -8118,13 +8118,13 @@
         <v>62</v>
       </c>
       <c r="K138" s="2" t="n">
-        <v>369</v>
+        <v>359</v>
       </c>
       <c r="L138" s="2" t="n">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="M138" s="2" t="n">
-        <v>665</v>
+        <v>645</v>
       </c>
       <c r="N138" s="4" t="inlineStr">
         <is>
@@ -8232,13 +8232,13 @@
         <v>47</v>
       </c>
       <c r="K140" s="2" t="n">
-        <v>228</v>
+        <v>441</v>
       </c>
       <c r="L140" s="2" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="M140" s="2" t="n">
-        <v>297</v>
+        <v>507</v>
       </c>
       <c r="N140" s="4" t="inlineStr">
         <is>
@@ -8346,13 +8346,13 @@
         <v>43</v>
       </c>
       <c r="K142" s="2" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="L142" s="2" t="n">
         <v>2</v>
       </c>
       <c r="M142" s="2" t="n">
-        <v>74</v>
+        <v>45</v>
       </c>
       <c r="N142" s="4" t="inlineStr">
         <is>
@@ -8805,10 +8805,10 @@
         <v>364</v>
       </c>
       <c r="L150" s="2" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M150" s="2" t="n">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="N150" s="6" t="inlineStr">
         <is>
@@ -9888,10 +9888,10 @@
         <v>139</v>
       </c>
       <c r="L169" s="2" t="n">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="M169" s="2" t="n">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="N169" s="4" t="inlineStr">
         <is>
@@ -10116,10 +10116,10 @@
         <v>68</v>
       </c>
       <c r="L173" s="2" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="M173" s="2" t="n">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="N173" s="4" t="inlineStr">
         <is>
@@ -10230,10 +10230,10 @@
         <v>22</v>
       </c>
       <c r="L175" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M175" s="2" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N175" s="4" t="inlineStr">
         <is>
@@ -11367,13 +11367,13 @@
         <v>187</v>
       </c>
       <c r="K195" s="2" t="n">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="L195" s="2" t="n">
         <v>149</v>
       </c>
       <c r="M195" s="2" t="n">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="N195" s="4" t="inlineStr">
         <is>
@@ -11766,13 +11766,13 @@
         <v>64</v>
       </c>
       <c r="K202" s="2" t="n">
-        <v>377</v>
+        <v>352</v>
       </c>
       <c r="L202" s="2" t="n">
         <v>299</v>
       </c>
       <c r="M202" s="2" t="n">
-        <v>740</v>
+        <v>715</v>
       </c>
       <c r="N202" s="4" t="inlineStr">
         <is>
@@ -11823,13 +11823,13 @@
         <v>167</v>
       </c>
       <c r="K203" s="2" t="n">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="L203" s="2" t="n">
         <v>50</v>
       </c>
       <c r="M203" s="2" t="n">
-        <v>295</v>
+        <v>275</v>
       </c>
       <c r="N203" s="4" t="inlineStr">
         <is>
@@ -11994,13 +11994,13 @@
         <v>182</v>
       </c>
       <c r="K206" s="2" t="n">
-        <v>302</v>
+        <v>288</v>
       </c>
       <c r="L206" s="2" t="n">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="M206" s="2" t="n">
-        <v>701</v>
+        <v>686</v>
       </c>
       <c r="N206" s="4" t="inlineStr">
         <is>
@@ -12051,13 +12051,13 @@
         <v>40</v>
       </c>
       <c r="K207" s="2" t="n">
-        <v>292</v>
+        <v>261</v>
       </c>
       <c r="L207" s="2" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="M207" s="2" t="n">
-        <v>342</v>
+        <v>331</v>
       </c>
       <c r="N207" s="4" t="inlineStr">
         <is>
@@ -12165,13 +12165,13 @@
         <v>111</v>
       </c>
       <c r="K209" s="2" t="n">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="L209" s="2" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="M209" s="2" t="n">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="N209" s="4" t="inlineStr">
         <is>
@@ -12336,13 +12336,13 @@
         <v>45</v>
       </c>
       <c r="K212" s="2" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L212" s="2" t="n">
         <v>53</v>
       </c>
       <c r="M212" s="2" t="n">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="N212" s="4" t="inlineStr">
         <is>
@@ -12792,13 +12792,13 @@
         <v>0</v>
       </c>
       <c r="K220" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L220" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M220" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N220" s="5" t="inlineStr">
         <is>
@@ -12846,7 +12846,7 @@
         </is>
       </c>
       <c r="J221" s="2" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="K221" s="2" t="n">
         <v>15</v>
@@ -12855,11 +12855,11 @@
         <v>6</v>
       </c>
       <c r="M221" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="N221" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>21</v>
+      </c>
+      <c r="N221" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O221" s="2" t="n">
@@ -13419,13 +13419,13 @@
         <v>396</v>
       </c>
       <c r="K231" s="2" t="n">
-        <v>327</v>
+        <v>317</v>
       </c>
       <c r="L231" s="2" t="n">
         <v>691</v>
       </c>
       <c r="M231" s="2" t="n">
-        <v>1414</v>
+        <v>1404</v>
       </c>
       <c r="N231" s="4" t="inlineStr">
         <is>
@@ -13530,10 +13530,10 @@
         </is>
       </c>
       <c r="J233" s="2" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="K233" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L233" s="2" t="n">
         <v>0</v>
@@ -13590,13 +13590,13 @@
         <v>1</v>
       </c>
       <c r="K234" s="2" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="L234" s="2" t="n">
         <v>11</v>
       </c>
       <c r="M234" s="2" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="N234" s="6" t="inlineStr">
         <is>
@@ -14217,13 +14217,13 @@
         <v>0</v>
       </c>
       <c r="K245" s="2" t="n">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="L245" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M245" s="2" t="n">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="N245" s="6" t="inlineStr">
         <is>
@@ -14790,10 +14790,10 @@
         <v>0</v>
       </c>
       <c r="L255" s="2" t="n">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="M255" s="2" t="n">
-        <v>199</v>
+        <v>184</v>
       </c>
       <c r="N255" s="4" t="inlineStr">
         <is>
@@ -14841,16 +14841,16 @@
         </is>
       </c>
       <c r="J256" s="2" t="n">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="K256" s="2" t="n">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="L256" s="2" t="n">
         <v>129</v>
       </c>
       <c r="M256" s="2" t="n">
-        <v>540</v>
+        <v>518</v>
       </c>
       <c r="N256" s="4" t="inlineStr">
         <is>
@@ -15015,13 +15015,13 @@
         <v>82</v>
       </c>
       <c r="K259" s="2" t="n">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="L259" s="2" t="n">
         <v>190</v>
       </c>
       <c r="M259" s="2" t="n">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="N259" s="4" t="inlineStr">
         <is>
@@ -15129,13 +15129,13 @@
         <v>29</v>
       </c>
       <c r="K261" s="2" t="n">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="L261" s="2" t="n">
         <v>7</v>
       </c>
       <c r="M261" s="2" t="n">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="N261" s="4" t="inlineStr">
         <is>
@@ -15243,13 +15243,13 @@
         <v>71</v>
       </c>
       <c r="K263" s="2" t="n">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L263" s="2" t="n">
         <v>68</v>
       </c>
       <c r="M263" s="2" t="n">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="N263" s="4" t="inlineStr">
         <is>
@@ -15753,7 +15753,7 @@
         </is>
       </c>
       <c r="J272" s="2" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K272" s="2" t="n">
         <v>0</v>
@@ -15762,7 +15762,7 @@
         <v>40</v>
       </c>
       <c r="M272" s="2" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="N272" s="4" t="inlineStr">
         <is>
@@ -15813,13 +15813,13 @@
         <v>39</v>
       </c>
       <c r="K273" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L273" s="2" t="n">
         <v>7</v>
       </c>
       <c r="M273" s="2" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="N273" s="4" t="inlineStr">
         <is>
@@ -15873,10 +15873,10 @@
         <v>205</v>
       </c>
       <c r="L274" s="2" t="n">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="M274" s="2" t="n">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="N274" s="4" t="inlineStr">
         <is>
@@ -16443,10 +16443,10 @@
         <v>328</v>
       </c>
       <c r="L284" s="2" t="n">
-        <v>82</v>
+        <v>238</v>
       </c>
       <c r="M284" s="2" t="n">
-        <v>437</v>
+        <v>593</v>
       </c>
       <c r="N284" s="4" t="inlineStr">
         <is>
@@ -16956,10 +16956,10 @@
         <v>5</v>
       </c>
       <c r="L293" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M293" s="2" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="N293" s="4" t="inlineStr">
         <is>
@@ -17409,13 +17409,13 @@
         <v>50</v>
       </c>
       <c r="K301" s="2" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="L301" s="2" t="n">
         <v>77</v>
       </c>
       <c r="M301" s="2" t="n">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="N301" s="4" t="inlineStr">
         <is>
@@ -17523,13 +17523,13 @@
         <v>26</v>
       </c>
       <c r="K303" s="2" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L303" s="2" t="n">
         <v>37</v>
       </c>
       <c r="M303" s="2" t="n">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="N303" s="4" t="inlineStr">
         <is>
@@ -17697,10 +17697,10 @@
         <v>24</v>
       </c>
       <c r="L306" s="2" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="M306" s="2" t="n">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="N306" s="4" t="inlineStr">
         <is>
@@ -17979,13 +17979,13 @@
         <v>12</v>
       </c>
       <c r="K311" s="2" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L311" s="2" t="n">
         <v>48</v>
       </c>
       <c r="M311" s="2" t="n">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="N311" s="4" t="inlineStr">
         <is>
@@ -18036,13 +18036,13 @@
         <v>169</v>
       </c>
       <c r="K312" s="2" t="n">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="L312" s="2" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="M312" s="2" t="n">
-        <v>422</v>
+        <v>409</v>
       </c>
       <c r="N312" s="4" t="inlineStr">
         <is>
@@ -18147,7 +18147,7 @@
         </is>
       </c>
       <c r="J314" s="2" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="K314" s="2" t="n">
         <v>60</v>
@@ -18156,11 +18156,11 @@
         <v>0</v>
       </c>
       <c r="M314" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="N314" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>69</v>
+      </c>
+      <c r="N314" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O314" s="2" t="n">
@@ -18606,13 +18606,13 @@
         <v>115</v>
       </c>
       <c r="K322" s="2" t="n">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="L322" s="2" t="n">
         <v>47</v>
       </c>
       <c r="M322" s="2" t="n">
-        <v>288</v>
+        <v>276</v>
       </c>
       <c r="N322" s="4" t="inlineStr">
         <is>
@@ -18834,13 +18834,13 @@
         <v>44</v>
       </c>
       <c r="K326" s="2" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="L326" s="2" t="n">
         <v>59</v>
       </c>
       <c r="M326" s="2" t="n">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="N326" s="4" t="inlineStr">
         <is>
@@ -19290,13 +19290,13 @@
         <v>7</v>
       </c>
       <c r="K334" s="2" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="L334" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M334" s="2" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="N334" s="6" t="inlineStr">
         <is>
@@ -19347,13 +19347,13 @@
         <v>56</v>
       </c>
       <c r="K335" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="L335" s="2" t="n">
         <v>83</v>
       </c>
       <c r="M335" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="N335" s="4" t="inlineStr">
         <is>
@@ -19407,10 +19407,10 @@
         <v>87</v>
       </c>
       <c r="L336" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="M336" s="2" t="n">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="N336" s="4" t="inlineStr">
         <is>
@@ -19518,13 +19518,13 @@
         <v>92</v>
       </c>
       <c r="K338" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L338" s="2" t="n">
         <v>71</v>
       </c>
       <c r="M338" s="2" t="n">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="N338" s="4" t="inlineStr">
         <is>
@@ -19977,10 +19977,10 @@
         <v>286</v>
       </c>
       <c r="L346" s="2" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="M346" s="2" t="n">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="N346" s="4" t="inlineStr">
         <is>
@@ -20028,20 +20028,20 @@
         </is>
       </c>
       <c r="J347" s="2" t="n">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="K347" s="2" t="n">
-        <v>247</v>
+        <v>135</v>
       </c>
       <c r="L347" s="2" t="n">
         <v>119</v>
       </c>
       <c r="M347" s="2" t="n">
-        <v>370</v>
-      </c>
-      <c r="N347" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>356</v>
+      </c>
+      <c r="N347" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O347" s="2" t="n">
@@ -20319,10 +20319,10 @@
         <v>282</v>
       </c>
       <c r="L352" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="M352" s="2" t="n">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="N352" s="4" t="inlineStr">
         <is>
@@ -20370,7 +20370,7 @@
         </is>
       </c>
       <c r="J353" s="2" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K353" s="2" t="n">
         <v>183</v>
@@ -20379,7 +20379,7 @@
         <v>26</v>
       </c>
       <c r="M353" s="2" t="n">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="N353" s="4" t="inlineStr">
         <is>
@@ -21231,10 +21231,10 @@
         <v>2</v>
       </c>
       <c r="L368" s="2" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="M368" s="2" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="N368" s="6" t="inlineStr">
         <is>
@@ -21285,13 +21285,13 @@
         <v>3</v>
       </c>
       <c r="K369" s="2" t="n">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="L369" s="2" t="n">
         <v>7</v>
       </c>
       <c r="M369" s="2" t="n">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="N369" s="6" t="inlineStr">
         <is>
@@ -21345,10 +21345,10 @@
         <v>51</v>
       </c>
       <c r="L370" s="2" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M370" s="2" t="n">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="N370" s="4" t="inlineStr">
         <is>
@@ -21855,13 +21855,13 @@
         <v>0</v>
       </c>
       <c r="K379" s="2" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L379" s="2" t="n">
         <v>22</v>
       </c>
       <c r="M379" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="N379" s="6" t="inlineStr">
         <is>
@@ -21966,7 +21966,7 @@
         </is>
       </c>
       <c r="J381" s="2" t="n">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="K381" s="2" t="n">
         <v>151</v>
@@ -21975,7 +21975,7 @@
         <v>94</v>
       </c>
       <c r="M381" s="2" t="n">
-        <v>350</v>
+        <v>338</v>
       </c>
       <c r="N381" s="4" t="inlineStr">
         <is>
@@ -22764,20 +22764,20 @@
         </is>
       </c>
       <c r="J395" s="2" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="K395" s="2" t="n">
-        <v>140</v>
+        <v>104</v>
       </c>
       <c r="L395" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M395" s="2" t="n">
-        <v>140</v>
-      </c>
-      <c r="N395" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>132</v>
+      </c>
+      <c r="N395" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O395" s="2" t="n">
@@ -22881,13 +22881,13 @@
         <v>104</v>
       </c>
       <c r="K397" s="2" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="L397" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M397" s="2" t="n">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="N397" s="4" t="inlineStr">
         <is>
@@ -23047,7 +23047,7 @@
         </is>
       </c>
       <c r="J400" s="2" t="n">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="K400" s="2" t="n">
         <v>0</v>
@@ -23056,7 +23056,7 @@
         <v>794</v>
       </c>
       <c r="M400" s="2" t="n">
-        <v>937</v>
+        <v>927</v>
       </c>
       <c r="N400" s="4" t="inlineStr">
         <is>
@@ -23270,13 +23270,13 @@
         <v>178</v>
       </c>
       <c r="K404" s="2" t="n">
-        <v>187</v>
+        <v>112</v>
       </c>
       <c r="L404" s="2" t="n">
         <v>54</v>
       </c>
       <c r="M404" s="2" t="n">
-        <v>419</v>
+        <v>344</v>
       </c>
       <c r="N404" s="4" t="inlineStr">
         <is>
@@ -23894,16 +23894,16 @@
         </is>
       </c>
       <c r="J415" s="2" t="n">
-        <v>198</v>
+        <v>138</v>
       </c>
       <c r="K415" s="2" t="n">
-        <v>1111</v>
+        <v>1091</v>
       </c>
       <c r="L415" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M415" s="2" t="n">
-        <v>1309</v>
+        <v>1229</v>
       </c>
       <c r="N415" s="4" t="inlineStr">
         <is>
@@ -23954,13 +23954,13 @@
         <v>242</v>
       </c>
       <c r="K416" s="2" t="n">
-        <v>1904</v>
+        <v>1899</v>
       </c>
       <c r="L416" s="2" t="n">
         <v>655</v>
       </c>
       <c r="M416" s="2" t="n">
-        <v>2801</v>
+        <v>2796</v>
       </c>
       <c r="N416" s="4" t="inlineStr">
         <is>
@@ -24011,13 +24011,13 @@
         <v>179</v>
       </c>
       <c r="K417" s="2" t="n">
-        <v>659</v>
+        <v>654</v>
       </c>
       <c r="L417" s="2" t="n">
         <v>81</v>
       </c>
       <c r="M417" s="2" t="n">
-        <v>919</v>
+        <v>914</v>
       </c>
       <c r="N417" s="4" t="inlineStr">
         <is>
@@ -24125,13 +24125,13 @@
         <v>279</v>
       </c>
       <c r="K419" s="2" t="n">
-        <v>881</v>
+        <v>869</v>
       </c>
       <c r="L419" s="2" t="n">
         <v>7</v>
       </c>
       <c r="M419" s="2" t="n">
-        <v>1167</v>
+        <v>1155</v>
       </c>
       <c r="N419" s="4" t="inlineStr">
         <is>
@@ -24293,7 +24293,7 @@
         </is>
       </c>
       <c r="J422" s="2" t="n">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="K422" s="2" t="n">
         <v>484</v>
@@ -24302,7 +24302,7 @@
         <v>256</v>
       </c>
       <c r="M422" s="2" t="n">
-        <v>881</v>
+        <v>861</v>
       </c>
       <c r="N422" s="4" t="inlineStr">
         <is>
@@ -24581,13 +24581,13 @@
         <v>85</v>
       </c>
       <c r="K427" s="2" t="n">
-        <v>642</v>
+        <v>348</v>
       </c>
       <c r="L427" s="2" t="n">
         <v>121</v>
       </c>
       <c r="M427" s="2" t="n">
-        <v>848</v>
+        <v>554</v>
       </c>
       <c r="N427" s="4" t="inlineStr">
         <is>
@@ -24752,13 +24752,13 @@
         <v>179</v>
       </c>
       <c r="K430" s="2" t="n">
-        <v>184</v>
+        <v>143</v>
       </c>
       <c r="L430" s="2" t="n">
         <v>224</v>
       </c>
       <c r="M430" s="2" t="n">
-        <v>587</v>
+        <v>546</v>
       </c>
       <c r="N430" s="4" t="inlineStr">
         <is>
@@ -24980,13 +24980,13 @@
         <v>141</v>
       </c>
       <c r="K434" s="2" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="L434" s="2" t="n">
         <v>88</v>
       </c>
       <c r="M434" s="2" t="n">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="N434" s="4" t="inlineStr">
         <is>
@@ -25205,7 +25205,7 @@
         </is>
       </c>
       <c r="J438" s="2" t="n">
-        <v>331</v>
+        <v>232</v>
       </c>
       <c r="K438" s="2" t="n">
         <v>341</v>
@@ -25214,7 +25214,7 @@
         <v>81</v>
       </c>
       <c r="M438" s="2" t="n">
-        <v>753</v>
+        <v>654</v>
       </c>
       <c r="N438" s="4" t="inlineStr">
         <is>
@@ -25550,13 +25550,13 @@
         <v>167</v>
       </c>
       <c r="K444" s="2" t="n">
-        <v>85</v>
+        <v>241</v>
       </c>
       <c r="L444" s="2" t="n">
         <v>95</v>
       </c>
       <c r="M444" s="2" t="n">
-        <v>347</v>
+        <v>503</v>
       </c>
       <c r="N444" s="4" t="inlineStr">
         <is>
@@ -25661,16 +25661,16 @@
         </is>
       </c>
       <c r="J446" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K446" s="2" t="n">
-        <v>112</v>
+        <v>91</v>
       </c>
       <c r="L446" s="2" t="n">
         <v>38</v>
       </c>
       <c r="M446" s="2" t="n">
-        <v>150</v>
+        <v>132</v>
       </c>
       <c r="N446" s="6" t="inlineStr">
         <is>
@@ -25952,10 +25952,10 @@
         <v>54</v>
       </c>
       <c r="L451" s="2" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="M451" s="2" t="n">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="N451" s="4" t="inlineStr">
         <is>
@@ -26009,10 +26009,10 @@
         <v>1</v>
       </c>
       <c r="L452" s="2" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="M452" s="2" t="n">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="N452" s="4" t="inlineStr">
         <is>
@@ -26288,16 +26288,16 @@
         </is>
       </c>
       <c r="J457" s="2" t="n">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="K457" s="2" t="n">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="L457" s="2" t="n">
         <v>266</v>
       </c>
       <c r="M457" s="2" t="n">
-        <v>789</v>
+        <v>775</v>
       </c>
       <c r="N457" s="4" t="inlineStr">
         <is>
@@ -26405,13 +26405,13 @@
         <v>42</v>
       </c>
       <c r="K459" s="2" t="n">
-        <v>228</v>
+        <v>204</v>
       </c>
       <c r="L459" s="2" t="n">
         <v>205</v>
       </c>
       <c r="M459" s="2" t="n">
-        <v>475</v>
+        <v>451</v>
       </c>
       <c r="N459" s="4" t="inlineStr">
         <is>
@@ -26462,13 +26462,13 @@
         <v>1</v>
       </c>
       <c r="K460" s="2" t="n">
-        <v>464</v>
+        <v>359</v>
       </c>
       <c r="L460" s="2" t="n">
-        <v>322</v>
+        <v>292</v>
       </c>
       <c r="M460" s="2" t="n">
-        <v>787</v>
+        <v>652</v>
       </c>
       <c r="N460" s="6" t="inlineStr">
         <is>
@@ -26519,13 +26519,13 @@
         <v>26</v>
       </c>
       <c r="K461" s="2" t="n">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="L461" s="2" t="n">
         <v>24</v>
       </c>
       <c r="M461" s="2" t="n">
-        <v>265</v>
+        <v>250</v>
       </c>
       <c r="N461" s="4" t="inlineStr">
         <is>
@@ -26975,13 +26975,13 @@
         <v>11</v>
       </c>
       <c r="K469" s="2" t="n">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="L469" s="2" t="n">
         <v>28</v>
       </c>
       <c r="M469" s="2" t="n">
-        <v>120</v>
+        <v>108</v>
       </c>
       <c r="N469" s="4" t="inlineStr">
         <is>
@@ -27029,16 +27029,16 @@
         </is>
       </c>
       <c r="J470" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K470" s="2" t="n">
         <v>117</v>
       </c>
       <c r="L470" s="2" t="n">
-        <v>126</v>
+        <v>96</v>
       </c>
       <c r="M470" s="2" t="n">
-        <v>243</v>
+        <v>221</v>
       </c>
       <c r="N470" s="6" t="inlineStr">
         <is>
@@ -27089,13 +27089,13 @@
         <v>25</v>
       </c>
       <c r="K471" s="2" t="n">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="L471" s="2" t="n">
         <v>77</v>
       </c>
       <c r="M471" s="2" t="n">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="N471" s="4" t="inlineStr">
         <is>
@@ -27488,13 +27488,13 @@
         <v>1</v>
       </c>
       <c r="K478" s="2" t="n">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="L478" s="2" t="n">
         <v>3</v>
       </c>
       <c r="M478" s="2" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="N478" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update inventario_expandido.xlsx - 16/10/2026
</commit_message>
<xml_diff>
--- a/inventario_expandido.xlsx
+++ b/inventario_expandido.xlsx
@@ -785,13 +785,13 @@
         <v>298</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>391</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
@@ -898,10 +898,10 @@
         <v>92</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="J20" s="2" t="n">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="K20" s="2" t="n">
         <v>116</v>
@@ -1604,7 +1604,7 @@
         <v>86</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
@@ -1701,10 +1701,10 @@
         </is>
       </c>
       <c r="J22" s="2" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="L22" s="2" t="n">
         <v>0</v>
@@ -2019,16 +2019,16 @@
         </is>
       </c>
       <c r="J28" s="2" t="n">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>540</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>1196</v>
+        <v>1194</v>
       </c>
       <c r="N28" s="4" t="inlineStr">
         <is>
@@ -2348,13 +2348,13 @@
         <v>348</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>417</v>
+        <v>405</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>183</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>948</v>
+        <v>936</v>
       </c>
       <c r="N34" s="4" t="inlineStr">
         <is>
@@ -2458,13 +2458,13 @@
         <v>66</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N36" s="4" t="inlineStr">
         <is>
@@ -2678,13 +2678,13 @@
         <v>57</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>607</v>
+        <v>597</v>
       </c>
       <c r="L40" s="2" t="n">
         <v>174</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>838</v>
+        <v>828</v>
       </c>
       <c r="N40" s="4" t="inlineStr">
         <is>
@@ -2788,13 +2788,13 @@
         <v>142</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>86</v>
       </c>
       <c r="M42" s="2" t="n">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="N42" s="4" t="inlineStr">
         <is>
@@ -3060,7 +3060,7 @@
         </is>
       </c>
       <c r="J47" s="2" t="n">
-        <v>166</v>
+        <v>121</v>
       </c>
       <c r="K47" s="2" t="n">
         <v>153</v>
@@ -3069,7 +3069,7 @@
         <v>147</v>
       </c>
       <c r="M47" s="2" t="n">
-        <v>466</v>
+        <v>421</v>
       </c>
       <c r="N47" s="4" t="inlineStr">
         <is>
@@ -3338,13 +3338,13 @@
         <v>2</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="L52" s="2" t="n">
         <v>17</v>
       </c>
       <c r="M52" s="2" t="n">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="N52" s="6" t="inlineStr">
         <is>
@@ -3778,13 +3778,13 @@
         <v>40</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L60" s="2" t="n">
         <v>28</v>
       </c>
       <c r="M60" s="2" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="N60" s="4" t="inlineStr">
         <is>
@@ -3833,13 +3833,13 @@
         <v>61</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="L61" s="2" t="n">
         <v>20</v>
       </c>
       <c r="M61" s="2" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N61" s="4" t="inlineStr">
         <is>
@@ -3940,10 +3940,10 @@
         </is>
       </c>
       <c r="J63" s="2" t="n">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>108</v>
+        <v>83</v>
       </c>
       <c r="L63" s="2" t="n">
         <v>53</v>
@@ -4823,13 +4823,13 @@
         <v>87</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="L79" s="2" t="n">
         <v>170</v>
       </c>
       <c r="M79" s="2" t="n">
-        <v>270</v>
+        <v>257</v>
       </c>
       <c r="N79" s="4" t="inlineStr">
         <is>
@@ -5535,7 +5535,7 @@
         </is>
       </c>
       <c r="J92" s="2" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>506</v>
@@ -5544,7 +5544,7 @@
         <v>0</v>
       </c>
       <c r="M92" s="2" t="n">
-        <v>520</v>
+        <v>516</v>
       </c>
       <c r="N92" s="4" t="inlineStr">
         <is>
@@ -5590,7 +5590,7 @@
         </is>
       </c>
       <c r="J93" s="2" t="n">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>11</v>
@@ -5599,7 +5599,7 @@
         <v>103</v>
       </c>
       <c r="M93" s="2" t="n">
-        <v>330</v>
+        <v>314</v>
       </c>
       <c r="N93" s="4" t="inlineStr">
         <is>
@@ -6864,13 +6864,13 @@
         <v>0</v>
       </c>
       <c r="K116" s="2" t="n">
-        <v>66</v>
+        <v>16</v>
       </c>
       <c r="L116" s="2" t="n">
-        <v>46</v>
+        <v>94</v>
       </c>
       <c r="M116" s="2" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="N116" s="6" t="inlineStr">
         <is>
@@ -8058,16 +8058,16 @@
         </is>
       </c>
       <c r="J137" s="2" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="K137" s="2" t="n">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="L137" s="2" t="n">
         <v>187</v>
       </c>
       <c r="M137" s="2" t="n">
-        <v>430</v>
+        <v>422</v>
       </c>
       <c r="N137" s="4" t="inlineStr">
         <is>
@@ -8118,13 +8118,13 @@
         <v>62</v>
       </c>
       <c r="K138" s="2" t="n">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="L138" s="2" t="n">
-        <v>224</v>
+        <v>184</v>
       </c>
       <c r="M138" s="2" t="n">
-        <v>645</v>
+        <v>603</v>
       </c>
       <c r="N138" s="4" t="inlineStr">
         <is>
@@ -8403,13 +8403,13 @@
         <v>122</v>
       </c>
       <c r="K143" s="2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L143" s="2" t="n">
         <v>32</v>
       </c>
       <c r="M143" s="2" t="n">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="N143" s="4" t="inlineStr">
         <is>
@@ -8802,13 +8802,13 @@
         <v>0</v>
       </c>
       <c r="K150" s="2" t="n">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="L150" s="2" t="n">
         <v>16</v>
       </c>
       <c r="M150" s="2" t="n">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="N150" s="6" t="inlineStr">
         <is>
@@ -9885,10 +9885,10 @@
         <v>101</v>
       </c>
       <c r="K169" s="2" t="n">
-        <v>139</v>
+        <v>99</v>
       </c>
       <c r="L169" s="2" t="n">
-        <v>79</v>
+        <v>119</v>
       </c>
       <c r="M169" s="2" t="n">
         <v>319</v>
@@ -10056,13 +10056,13 @@
         <v>256</v>
       </c>
       <c r="K172" s="2" t="n">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="L172" s="2" t="n">
         <v>319</v>
       </c>
       <c r="M172" s="2" t="n">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="N172" s="4" t="inlineStr">
         <is>
@@ -10110,16 +10110,16 @@
         </is>
       </c>
       <c r="J173" s="2" t="n">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="K173" s="2" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="L173" s="2" t="n">
         <v>80</v>
       </c>
       <c r="M173" s="2" t="n">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="N173" s="4" t="inlineStr">
         <is>
@@ -10626,17 +10626,17 @@
         <v>9</v>
       </c>
       <c r="K182" s="2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="L182" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M182" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="N182" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>18</v>
+      </c>
+      <c r="N182" s="5" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
         </is>
       </c>
       <c r="O182" s="2" t="n">
@@ -11139,13 +11139,13 @@
         <v>52</v>
       </c>
       <c r="K191" s="2" t="n">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="L191" s="2" t="n">
         <v>42</v>
       </c>
       <c r="M191" s="2" t="n">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="N191" s="4" t="inlineStr">
         <is>
@@ -11253,13 +11253,13 @@
         <v>0</v>
       </c>
       <c r="K193" s="2" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="L193" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M193" s="2" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="N193" s="6" t="inlineStr">
         <is>
@@ -11424,13 +11424,13 @@
         <v>204</v>
       </c>
       <c r="K196" s="2" t="n">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="L196" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M196" s="2" t="n">
-        <v>272</v>
+        <v>240</v>
       </c>
       <c r="N196" s="4" t="inlineStr">
         <is>
@@ -11994,13 +11994,13 @@
         <v>182</v>
       </c>
       <c r="K206" s="2" t="n">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="L206" s="2" t="n">
         <v>216</v>
       </c>
       <c r="M206" s="2" t="n">
-        <v>686</v>
+        <v>683</v>
       </c>
       <c r="N206" s="4" t="inlineStr">
         <is>
@@ -12105,7 +12105,7 @@
         </is>
       </c>
       <c r="J208" s="2" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="K208" s="2" t="n">
         <v>30</v>
@@ -12114,7 +12114,7 @@
         <v>76</v>
       </c>
       <c r="M208" s="2" t="n">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="N208" s="4" t="inlineStr">
         <is>
@@ -12165,13 +12165,13 @@
         <v>111</v>
       </c>
       <c r="K209" s="2" t="n">
-        <v>123</v>
+        <v>88</v>
       </c>
       <c r="L209" s="2" t="n">
         <v>39</v>
       </c>
       <c r="M209" s="2" t="n">
-        <v>273</v>
+        <v>238</v>
       </c>
       <c r="N209" s="4" t="inlineStr">
         <is>
@@ -12450,13 +12450,13 @@
         <v>120</v>
       </c>
       <c r="K214" s="2" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="L214" s="2" t="n">
         <v>80</v>
       </c>
       <c r="M214" s="2" t="n">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="N214" s="4" t="inlineStr">
         <is>
@@ -12732,10 +12732,10 @@
         </is>
       </c>
       <c r="J219" s="2" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="K219" s="2" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="L219" s="2" t="n">
         <v>2</v>
@@ -12849,17 +12849,17 @@
         <v>0</v>
       </c>
       <c r="K221" s="2" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="L221" s="2" t="n">
         <v>6</v>
       </c>
       <c r="M221" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="N221" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>9</v>
+      </c>
+      <c r="N221" s="5" t="inlineStr">
+        <is>
+          <t>Sin stock</t>
         </is>
       </c>
       <c r="O221" s="2" t="n">
@@ -13020,13 +13020,13 @@
         <v>7</v>
       </c>
       <c r="K224" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="L224" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M224" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="N224" s="6" t="inlineStr">
         <is>
@@ -13533,13 +13533,13 @@
         <v>11</v>
       </c>
       <c r="K233" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L233" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M233" s="2" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="N233" s="4" t="inlineStr">
         <is>
@@ -13758,20 +13758,20 @@
         </is>
       </c>
       <c r="J237" s="2" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="K237" s="2" t="n">
-        <v>85</v>
+        <v>61</v>
       </c>
       <c r="L237" s="2" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="M237" s="2" t="n">
         <v>113</v>
       </c>
-      <c r="N237" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+      <c r="N237" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O237" s="2" t="n">
@@ -13935,10 +13935,10 @@
         <v>17</v>
       </c>
       <c r="L240" s="2" t="n">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="M240" s="2" t="n">
-        <v>108</v>
+        <v>84</v>
       </c>
       <c r="N240" s="4" t="inlineStr">
         <is>
@@ -14328,7 +14328,7 @@
         </is>
       </c>
       <c r="J247" s="2" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="K247" s="2" t="n">
         <v>81</v>
@@ -14337,11 +14337,11 @@
         <v>0</v>
       </c>
       <c r="M247" s="2" t="n">
-        <v>91</v>
-      </c>
-      <c r="N247" s="4" t="inlineStr">
-        <is>
-          <t>Stock</t>
+        <v>82</v>
+      </c>
+      <c r="N247" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O247" s="2" t="n">
@@ -14385,7 +14385,7 @@
         </is>
       </c>
       <c r="J248" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="K248" s="2" t="n">
         <v>0</v>
@@ -14394,7 +14394,7 @@
         <v>0</v>
       </c>
       <c r="M248" s="2" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="N248" s="4" t="inlineStr">
         <is>
@@ -14442,7 +14442,7 @@
         </is>
       </c>
       <c r="J249" s="2" t="n">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K249" s="2" t="n">
         <v>192</v>
@@ -14451,7 +14451,7 @@
         <v>182</v>
       </c>
       <c r="M249" s="2" t="n">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="N249" s="4" t="inlineStr">
         <is>
@@ -15015,13 +15015,13 @@
         <v>82</v>
       </c>
       <c r="K259" s="2" t="n">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="L259" s="2" t="n">
         <v>190</v>
       </c>
       <c r="M259" s="2" t="n">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="N259" s="4" t="inlineStr">
         <is>
@@ -15072,13 +15072,13 @@
         <v>139</v>
       </c>
       <c r="K260" s="2" t="n">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="L260" s="2" t="n">
         <v>30</v>
       </c>
       <c r="M260" s="2" t="n">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="N260" s="4" t="inlineStr">
         <is>
@@ -15129,13 +15129,13 @@
         <v>29</v>
       </c>
       <c r="K261" s="2" t="n">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="L261" s="2" t="n">
         <v>7</v>
       </c>
       <c r="M261" s="2" t="n">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="N261" s="4" t="inlineStr">
         <is>
@@ -15300,13 +15300,13 @@
         <v>94</v>
       </c>
       <c r="K264" s="2" t="n">
-        <v>96</v>
+        <v>46</v>
       </c>
       <c r="L264" s="2" t="n">
         <v>95</v>
       </c>
       <c r="M264" s="2" t="n">
-        <v>285</v>
+        <v>235</v>
       </c>
       <c r="N264" s="4" t="inlineStr">
         <is>
@@ -15411,7 +15411,7 @@
         </is>
       </c>
       <c r="J266" s="2" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="K266" s="2" t="n">
         <v>42</v>
@@ -15420,7 +15420,7 @@
         <v>73</v>
       </c>
       <c r="M266" s="2" t="n">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N266" s="4" t="inlineStr">
         <is>
@@ -15873,10 +15873,10 @@
         <v>205</v>
       </c>
       <c r="L274" s="2" t="n">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="M274" s="2" t="n">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="N274" s="4" t="inlineStr">
         <is>
@@ -16383,13 +16383,13 @@
         <v>81</v>
       </c>
       <c r="K283" s="2" t="n">
-        <v>17</v>
+        <v>70</v>
       </c>
       <c r="L283" s="2" t="n">
-        <v>73</v>
+        <v>3</v>
       </c>
       <c r="M283" s="2" t="n">
-        <v>171</v>
+        <v>154</v>
       </c>
       <c r="N283" s="4" t="inlineStr">
         <is>
@@ -16437,7 +16437,7 @@
         </is>
       </c>
       <c r="J284" s="2" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="K284" s="2" t="n">
         <v>328</v>
@@ -16446,7 +16446,7 @@
         <v>238</v>
       </c>
       <c r="M284" s="2" t="n">
-        <v>593</v>
+        <v>588</v>
       </c>
       <c r="N284" s="4" t="inlineStr">
         <is>
@@ -17349,20 +17349,20 @@
         </is>
       </c>
       <c r="J300" s="2" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="K300" s="2" t="n">
-        <v>246</v>
+        <v>134</v>
       </c>
       <c r="L300" s="2" t="n">
-        <v>11</v>
+        <v>81</v>
       </c>
       <c r="M300" s="2" t="n">
         <v>257</v>
       </c>
-      <c r="N300" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+      <c r="N300" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O300" s="2" t="n">
@@ -17523,13 +17523,13 @@
         <v>26</v>
       </c>
       <c r="K303" s="2" t="n">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="L303" s="2" t="n">
         <v>37</v>
       </c>
       <c r="M303" s="2" t="n">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="N303" s="4" t="inlineStr">
         <is>
@@ -17583,10 +17583,10 @@
         <v>169</v>
       </c>
       <c r="L304" s="2" t="n">
-        <v>140</v>
+        <v>242</v>
       </c>
       <c r="M304" s="2" t="n">
-        <v>439</v>
+        <v>541</v>
       </c>
       <c r="N304" s="4" t="inlineStr">
         <is>
@@ -17697,10 +17697,10 @@
         <v>24</v>
       </c>
       <c r="L306" s="2" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="M306" s="2" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="N306" s="4" t="inlineStr">
         <is>
@@ -17865,13 +17865,13 @@
         <v>38</v>
       </c>
       <c r="K309" s="2" t="n">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="L309" s="2" t="n">
         <v>48</v>
       </c>
       <c r="M309" s="2" t="n">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="N309" s="4" t="inlineStr">
         <is>
@@ -18264,13 +18264,13 @@
         <v>24</v>
       </c>
       <c r="K316" s="2" t="n">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="L316" s="2" t="n">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="M316" s="2" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="N316" s="4" t="inlineStr">
         <is>
@@ -18378,10 +18378,10 @@
         <v>11</v>
       </c>
       <c r="K318" s="2" t="n">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="L318" s="2" t="n">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="M318" s="2" t="n">
         <v>79</v>
@@ -18603,16 +18603,16 @@
         </is>
       </c>
       <c r="J322" s="2" t="n">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="K322" s="2" t="n">
-        <v>114</v>
+        <v>87</v>
       </c>
       <c r="L322" s="2" t="n">
         <v>47</v>
       </c>
       <c r="M322" s="2" t="n">
-        <v>276</v>
+        <v>235</v>
       </c>
       <c r="N322" s="4" t="inlineStr">
         <is>
@@ -18831,7 +18831,7 @@
         </is>
       </c>
       <c r="J326" s="2" t="n">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="K326" s="2" t="n">
         <v>47</v>
@@ -18840,7 +18840,7 @@
         <v>59</v>
       </c>
       <c r="M326" s="2" t="n">
-        <v>150</v>
+        <v>134</v>
       </c>
       <c r="N326" s="4" t="inlineStr">
         <is>
@@ -19002,10 +19002,10 @@
         </is>
       </c>
       <c r="J329" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K329" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L329" s="2" t="n">
         <v>0</v>
@@ -19350,10 +19350,10 @@
         <v>75</v>
       </c>
       <c r="L335" s="2" t="n">
-        <v>83</v>
+        <v>49</v>
       </c>
       <c r="M335" s="2" t="n">
-        <v>214</v>
+        <v>180</v>
       </c>
       <c r="N335" s="4" t="inlineStr">
         <is>
@@ -19521,10 +19521,10 @@
         <v>2</v>
       </c>
       <c r="L338" s="2" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="M338" s="2" t="n">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="N338" s="4" t="inlineStr">
         <is>
@@ -19572,7 +19572,7 @@
         </is>
       </c>
       <c r="J339" s="2" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K339" s="2" t="n">
         <v>197</v>
@@ -19581,7 +19581,7 @@
         <v>139</v>
       </c>
       <c r="M339" s="2" t="n">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="N339" s="4" t="inlineStr">
         <is>
@@ -19860,13 +19860,13 @@
         <v>83</v>
       </c>
       <c r="K344" s="2" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="L344" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="M344" s="2" t="n">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="N344" s="4" t="inlineStr">
         <is>
@@ -19971,7 +19971,7 @@
         </is>
       </c>
       <c r="J346" s="2" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K346" s="2" t="n">
         <v>286</v>
@@ -19980,7 +19980,7 @@
         <v>66</v>
       </c>
       <c r="M346" s="2" t="n">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="N346" s="4" t="inlineStr">
         <is>
@@ -20031,13 +20031,13 @@
         <v>102</v>
       </c>
       <c r="K347" s="2" t="n">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="L347" s="2" t="n">
         <v>119</v>
       </c>
       <c r="M347" s="2" t="n">
-        <v>356</v>
+        <v>345</v>
       </c>
       <c r="N347" s="4" t="inlineStr">
         <is>
@@ -20145,13 +20145,13 @@
         <v>99</v>
       </c>
       <c r="K349" s="2" t="n">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="L349" s="2" t="n">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="M349" s="2" t="n">
-        <v>537</v>
+        <v>521</v>
       </c>
       <c r="N349" s="4" t="inlineStr">
         <is>
@@ -20373,13 +20373,13 @@
         <v>51</v>
       </c>
       <c r="K353" s="2" t="n">
-        <v>183</v>
+        <v>151</v>
       </c>
       <c r="L353" s="2" t="n">
         <v>26</v>
       </c>
       <c r="M353" s="2" t="n">
-        <v>260</v>
+        <v>228</v>
       </c>
       <c r="N353" s="4" t="inlineStr">
         <is>
@@ -20433,10 +20433,10 @@
         <v>11</v>
       </c>
       <c r="L354" s="2" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M354" s="2" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="N354" s="4" t="inlineStr">
         <is>
@@ -20943,10 +20943,10 @@
         <v>0</v>
       </c>
       <c r="K363" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L363" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M363" s="2" t="n">
         <v>5</v>
@@ -21969,13 +21969,13 @@
         <v>93</v>
       </c>
       <c r="K381" s="2" t="n">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="L381" s="2" t="n">
         <v>94</v>
       </c>
       <c r="M381" s="2" t="n">
-        <v>338</v>
+        <v>328</v>
       </c>
       <c r="N381" s="4" t="inlineStr">
         <is>
@@ -22824,13 +22824,13 @@
         <v>0</v>
       </c>
       <c r="K396" s="2" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L396" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M396" s="2" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="N396" s="6" t="inlineStr">
         <is>
@@ -22878,7 +22878,7 @@
         </is>
       </c>
       <c r="J397" s="2" t="n">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="K397" s="2" t="n">
         <v>23</v>
@@ -22887,7 +22887,7 @@
         <v>0</v>
       </c>
       <c r="M397" s="2" t="n">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="N397" s="4" t="inlineStr">
         <is>
@@ -23270,13 +23270,13 @@
         <v>178</v>
       </c>
       <c r="K404" s="2" t="n">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="L404" s="2" t="n">
         <v>54</v>
       </c>
       <c r="M404" s="2" t="n">
-        <v>344</v>
+        <v>330</v>
       </c>
       <c r="N404" s="4" t="inlineStr">
         <is>
@@ -23384,13 +23384,13 @@
         <v>50</v>
       </c>
       <c r="K406" s="2" t="n">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="L406" s="2" t="n">
         <v>9</v>
       </c>
       <c r="M406" s="2" t="n">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="N406" s="4" t="inlineStr">
         <is>
@@ -24011,13 +24011,13 @@
         <v>179</v>
       </c>
       <c r="K417" s="2" t="n">
-        <v>654</v>
+        <v>624</v>
       </c>
       <c r="L417" s="2" t="n">
         <v>81</v>
       </c>
       <c r="M417" s="2" t="n">
-        <v>914</v>
+        <v>884</v>
       </c>
       <c r="N417" s="4" t="inlineStr">
         <is>
@@ -24125,13 +24125,13 @@
         <v>279</v>
       </c>
       <c r="K419" s="2" t="n">
-        <v>869</v>
+        <v>861</v>
       </c>
       <c r="L419" s="2" t="n">
         <v>7</v>
       </c>
       <c r="M419" s="2" t="n">
-        <v>1155</v>
+        <v>1147</v>
       </c>
       <c r="N419" s="4" t="inlineStr">
         <is>
@@ -24293,16 +24293,16 @@
         </is>
       </c>
       <c r="J422" s="2" t="n">
-        <v>121</v>
+        <v>102</v>
       </c>
       <c r="K422" s="2" t="n">
-        <v>484</v>
+        <v>472</v>
       </c>
       <c r="L422" s="2" t="n">
         <v>256</v>
       </c>
       <c r="M422" s="2" t="n">
-        <v>861</v>
+        <v>830</v>
       </c>
       <c r="N422" s="4" t="inlineStr">
         <is>
@@ -24410,13 +24410,13 @@
         <v>126</v>
       </c>
       <c r="K424" s="2" t="n">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="L424" s="2" t="n">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="M424" s="2" t="n">
-        <v>512</v>
+        <v>503</v>
       </c>
       <c r="N424" s="4" t="inlineStr">
         <is>
@@ -24581,13 +24581,13 @@
         <v>85</v>
       </c>
       <c r="K427" s="2" t="n">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="L427" s="2" t="n">
         <v>121</v>
       </c>
       <c r="M427" s="2" t="n">
-        <v>554</v>
+        <v>547</v>
       </c>
       <c r="N427" s="4" t="inlineStr">
         <is>
@@ -24752,13 +24752,13 @@
         <v>179</v>
       </c>
       <c r="K430" s="2" t="n">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="L430" s="2" t="n">
         <v>224</v>
       </c>
       <c r="M430" s="2" t="n">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="N430" s="4" t="inlineStr">
         <is>
@@ -24923,13 +24923,13 @@
         <v>225</v>
       </c>
       <c r="K433" s="2" t="n">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="L433" s="2" t="n">
         <v>31</v>
       </c>
       <c r="M433" s="2" t="n">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="N433" s="4" t="inlineStr">
         <is>
@@ -24980,13 +24980,13 @@
         <v>141</v>
       </c>
       <c r="K434" s="2" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="L434" s="2" t="n">
         <v>88</v>
       </c>
       <c r="M434" s="2" t="n">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="N434" s="4" t="inlineStr">
         <is>
@@ -25322,13 +25322,13 @@
         <v>0</v>
       </c>
       <c r="K440" s="2" t="n">
-        <v>287</v>
+        <v>261</v>
       </c>
       <c r="L440" s="2" t="n">
         <v>244</v>
       </c>
       <c r="M440" s="2" t="n">
-        <v>531</v>
+        <v>505</v>
       </c>
       <c r="N440" s="6" t="inlineStr">
         <is>
@@ -25493,13 +25493,13 @@
         <v>5</v>
       </c>
       <c r="K443" s="2" t="n">
-        <v>225</v>
+        <v>210</v>
       </c>
       <c r="L443" s="2" t="n">
         <v>210</v>
       </c>
       <c r="M443" s="2" t="n">
-        <v>440</v>
+        <v>425</v>
       </c>
       <c r="N443" s="6" t="inlineStr">
         <is>
@@ -25550,13 +25550,13 @@
         <v>167</v>
       </c>
       <c r="K444" s="2" t="n">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="L444" s="2" t="n">
         <v>95</v>
       </c>
       <c r="M444" s="2" t="n">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="N444" s="4" t="inlineStr">
         <is>
@@ -25895,10 +25895,10 @@
         <v>23</v>
       </c>
       <c r="L450" s="2" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="M450" s="2" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="N450" s="6" t="inlineStr">
         <is>
@@ -25952,10 +25952,10 @@
         <v>54</v>
       </c>
       <c r="L451" s="2" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="M451" s="2" t="n">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="N451" s="4" t="inlineStr">
         <is>
@@ -26120,13 +26120,13 @@
         <v>4</v>
       </c>
       <c r="K454" s="2" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="L454" s="2" t="n">
         <v>260</v>
       </c>
       <c r="M454" s="2" t="n">
-        <v>299</v>
+        <v>274</v>
       </c>
       <c r="N454" s="6" t="inlineStr">
         <is>
@@ -26177,13 +26177,13 @@
         <v>26</v>
       </c>
       <c r="K455" s="2" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="L455" s="2" t="n">
         <v>44</v>
       </c>
       <c r="M455" s="2" t="n">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="N455" s="4" t="inlineStr">
         <is>
@@ -26234,10 +26234,10 @@
         <v>0</v>
       </c>
       <c r="K456" s="2" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="L456" s="2" t="n">
-        <v>167</v>
+        <v>111</v>
       </c>
       <c r="M456" s="2" t="n">
         <v>167</v>
@@ -26291,13 +26291,13 @@
         <v>352</v>
       </c>
       <c r="K457" s="2" t="n">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="L457" s="2" t="n">
         <v>266</v>
       </c>
       <c r="M457" s="2" t="n">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="N457" s="4" t="inlineStr">
         <is>
@@ -26405,13 +26405,13 @@
         <v>42</v>
       </c>
       <c r="K459" s="2" t="n">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L459" s="2" t="n">
         <v>205</v>
       </c>
       <c r="M459" s="2" t="n">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="N459" s="4" t="inlineStr">
         <is>
@@ -26462,13 +26462,13 @@
         <v>1</v>
       </c>
       <c r="K460" s="2" t="n">
-        <v>359</v>
+        <v>339</v>
       </c>
       <c r="L460" s="2" t="n">
         <v>292</v>
       </c>
       <c r="M460" s="2" t="n">
-        <v>652</v>
+        <v>632</v>
       </c>
       <c r="N460" s="6" t="inlineStr">
         <is>
@@ -26576,13 +26576,13 @@
         <v>98</v>
       </c>
       <c r="K462" s="2" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="L462" s="2" t="n">
         <v>85</v>
       </c>
       <c r="M462" s="2" t="n">
-        <v>258</v>
+        <v>238</v>
       </c>
       <c r="N462" s="4" t="inlineStr">
         <is>
@@ -26975,13 +26975,13 @@
         <v>11</v>
       </c>
       <c r="K469" s="2" t="n">
-        <v>69</v>
+        <v>212</v>
       </c>
       <c r="L469" s="2" t="n">
         <v>28</v>
       </c>
       <c r="M469" s="2" t="n">
-        <v>108</v>
+        <v>251</v>
       </c>
       <c r="N469" s="4" t="inlineStr">
         <is>
@@ -28058,13 +28058,13 @@
         <v>0</v>
       </c>
       <c r="K488" s="2" t="n">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="L488" s="2" t="n">
         <v>323</v>
       </c>
       <c r="M488" s="2" t="n">
-        <v>496</v>
+        <v>490</v>
       </c>
       <c r="N488" s="6" t="inlineStr">
         <is>
@@ -28115,13 +28115,13 @@
         <v>0</v>
       </c>
       <c r="K489" s="2" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="L489" s="2" t="n">
         <v>28</v>
       </c>
       <c r="M489" s="2" t="n">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="N489" s="6" t="inlineStr">
         <is>
@@ -28172,13 +28172,13 @@
         <v>3</v>
       </c>
       <c r="K490" s="2" t="n">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="L490" s="2" t="n">
         <v>166</v>
       </c>
       <c r="M490" s="2" t="n">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="N490" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update inventario_expandido.xlsx - 23/10/2026
</commit_message>
<xml_diff>
--- a/inventario_expandido.xlsx
+++ b/inventario_expandido.xlsx
@@ -1383,16 +1383,16 @@
         </is>
       </c>
       <c r="J16" s="2" t="n">
-        <v>136</v>
+        <v>121</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>47</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>518</v>
+        <v>501</v>
       </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
@@ -1545,13 +1545,13 @@
         <v>0</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>2302</v>
+        <v>2301</v>
       </c>
       <c r="M19" s="2" t="n">
-        <v>2462</v>
+        <v>2451</v>
       </c>
       <c r="N19" s="6" t="inlineStr">
         <is>
@@ -1598,13 +1598,13 @@
         <v>92</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>86</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
@@ -2022,13 +2022,13 @@
         <v>319</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="L28" s="2" t="n">
         <v>335</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>1194</v>
+        <v>1191</v>
       </c>
       <c r="N28" s="4" t="inlineStr">
         <is>
@@ -2183,13 +2183,13 @@
         <v>318</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>944</v>
+        <v>924</v>
       </c>
       <c r="L31" s="2" t="n">
         <v>298</v>
       </c>
       <c r="M31" s="2" t="n">
-        <v>1560</v>
+        <v>1540</v>
       </c>
       <c r="N31" s="4" t="inlineStr">
         <is>
@@ -2345,16 +2345,16 @@
         </is>
       </c>
       <c r="J34" s="2" t="n">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>405</v>
+        <v>396</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>183</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>936</v>
+        <v>920</v>
       </c>
       <c r="N34" s="4" t="inlineStr">
         <is>
@@ -2568,13 +2568,13 @@
         <v>79</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="L38" s="2" t="n">
         <v>119</v>
       </c>
       <c r="M38" s="2" t="n">
-        <v>437</v>
+        <v>426</v>
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
@@ -2678,13 +2678,13 @@
         <v>57</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>597</v>
+        <v>584</v>
       </c>
       <c r="L40" s="2" t="n">
         <v>174</v>
       </c>
       <c r="M40" s="2" t="n">
-        <v>828</v>
+        <v>815</v>
       </c>
       <c r="N40" s="4" t="inlineStr">
         <is>
@@ -2733,13 +2733,13 @@
         <v>99</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="L41" s="2" t="n">
         <v>18</v>
       </c>
       <c r="M41" s="2" t="n">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="N41" s="4" t="inlineStr">
         <is>
@@ -3448,13 +3448,13 @@
         <v>73</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>30</v>
       </c>
       <c r="M54" s="2" t="n">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="N54" s="4" t="inlineStr">
         <is>
@@ -3561,10 +3561,10 @@
         <v>78</v>
       </c>
       <c r="L56" s="2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M56" s="2" t="n">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="N56" s="4" t="inlineStr">
         <is>
@@ -3668,13 +3668,13 @@
         <v>0</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M58" s="2" t="n">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="N58" s="6" t="inlineStr">
         <is>
@@ -3778,13 +3778,13 @@
         <v>40</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="L60" s="2" t="n">
         <v>28</v>
       </c>
       <c r="M60" s="2" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="N60" s="4" t="inlineStr">
         <is>
@@ -4548,13 +4548,13 @@
         <v>42</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="L74" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M74" s="2" t="n">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="N74" s="4" t="inlineStr">
         <is>
@@ -4603,13 +4603,13 @@
         <v>85</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="L75" s="2" t="n">
         <v>81</v>
       </c>
       <c r="M75" s="2" t="n">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="N75" s="4" t="inlineStr">
         <is>
@@ -4878,13 +4878,13 @@
         <v>80</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="L80" s="2" t="n">
         <v>64</v>
       </c>
       <c r="M80" s="2" t="n">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="N80" s="4" t="inlineStr">
         <is>
@@ -4988,13 +4988,13 @@
         <v>3</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="L82" s="2" t="n">
         <v>41</v>
       </c>
       <c r="M82" s="2" t="n">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="N82" s="6" t="inlineStr">
         <is>
@@ -5813,13 +5813,13 @@
         <v>45</v>
       </c>
       <c r="K97" s="2" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="L97" s="2" t="n">
         <v>5</v>
       </c>
       <c r="M97" s="2" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="N97" s="4" t="inlineStr">
         <is>
@@ -6418,13 +6418,13 @@
         <v>167</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="L108" s="2" t="n">
         <v>196</v>
       </c>
       <c r="M108" s="2" t="n">
-        <v>442</v>
+        <v>437</v>
       </c>
       <c r="N108" s="4" t="inlineStr">
         <is>
@@ -7266,10 +7266,10 @@
         <v>45</v>
       </c>
       <c r="L123" s="2" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="M123" s="2" t="n">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="N123" s="6" t="inlineStr">
         <is>
@@ -8061,13 +8061,13 @@
         <v>23</v>
       </c>
       <c r="K137" s="2" t="n">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="L137" s="2" t="n">
         <v>187</v>
       </c>
       <c r="M137" s="2" t="n">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="N137" s="4" t="inlineStr">
         <is>
@@ -8232,13 +8232,13 @@
         <v>47</v>
       </c>
       <c r="K140" s="2" t="n">
-        <v>441</v>
+        <v>431</v>
       </c>
       <c r="L140" s="2" t="n">
         <v>19</v>
       </c>
       <c r="M140" s="2" t="n">
-        <v>507</v>
+        <v>497</v>
       </c>
       <c r="N140" s="4" t="inlineStr">
         <is>
@@ -8346,13 +8346,13 @@
         <v>43</v>
       </c>
       <c r="K142" s="2" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="L142" s="2" t="n">
         <v>2</v>
       </c>
       <c r="M142" s="2" t="n">
-        <v>45</v>
+        <v>106</v>
       </c>
       <c r="N142" s="4" t="inlineStr">
         <is>
@@ -8802,13 +8802,13 @@
         <v>0</v>
       </c>
       <c r="K150" s="2" t="n">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="L150" s="2" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="M150" s="2" t="n">
-        <v>377</v>
+        <v>368</v>
       </c>
       <c r="N150" s="6" t="inlineStr">
         <is>
@@ -10002,10 +10002,10 @@
         <v>68</v>
       </c>
       <c r="L171" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M171" s="2" t="n">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="N171" s="4" t="inlineStr">
         <is>
@@ -10056,13 +10056,13 @@
         <v>256</v>
       </c>
       <c r="K172" s="2" t="n">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="L172" s="2" t="n">
         <v>319</v>
       </c>
       <c r="M172" s="2" t="n">
-        <v>783</v>
+        <v>780</v>
       </c>
       <c r="N172" s="4" t="inlineStr">
         <is>
@@ -10110,7 +10110,7 @@
         </is>
       </c>
       <c r="J173" s="2" t="n">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="K173" s="2" t="n">
         <v>66</v>
@@ -10119,7 +10119,7 @@
         <v>80</v>
       </c>
       <c r="M173" s="2" t="n">
-        <v>250</v>
+        <v>231</v>
       </c>
       <c r="N173" s="4" t="inlineStr">
         <is>
@@ -10395,10 +10395,10 @@
         </is>
       </c>
       <c r="J178" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K178" s="2" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="L178" s="2" t="n">
         <v>128</v>
@@ -11085,10 +11085,10 @@
         <v>66</v>
       </c>
       <c r="L190" s="2" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="M190" s="2" t="n">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="N190" s="4" t="inlineStr">
         <is>
@@ -11421,7 +11421,7 @@
         </is>
       </c>
       <c r="J196" s="2" t="n">
-        <v>204</v>
+        <v>159</v>
       </c>
       <c r="K196" s="2" t="n">
         <v>36</v>
@@ -11430,7 +11430,7 @@
         <v>0</v>
       </c>
       <c r="M196" s="2" t="n">
-        <v>240</v>
+        <v>195</v>
       </c>
       <c r="N196" s="4" t="inlineStr">
         <is>
@@ -11763,16 +11763,16 @@
         </is>
       </c>
       <c r="J202" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K202" s="2" t="n">
+        <v>277</v>
+      </c>
+      <c r="L202" s="2" t="n">
         <v>352</v>
       </c>
-      <c r="L202" s="2" t="n">
-        <v>299</v>
-      </c>
       <c r="M202" s="2" t="n">
-        <v>715</v>
+        <v>692</v>
       </c>
       <c r="N202" s="4" t="inlineStr">
         <is>
@@ -11820,7 +11820,7 @@
         </is>
       </c>
       <c r="J203" s="2" t="n">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="K203" s="2" t="n">
         <v>58</v>
@@ -11829,7 +11829,7 @@
         <v>50</v>
       </c>
       <c r="M203" s="2" t="n">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="N203" s="4" t="inlineStr">
         <is>
@@ -12168,10 +12168,10 @@
         <v>88</v>
       </c>
       <c r="L209" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="M209" s="2" t="n">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="N209" s="4" t="inlineStr">
         <is>
@@ -12564,13 +12564,13 @@
         <v>6</v>
       </c>
       <c r="K216" s="2" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="L216" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M216" s="2" t="n">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="N216" s="6" t="inlineStr">
         <is>
@@ -13134,13 +13134,13 @@
         <v>0</v>
       </c>
       <c r="K226" s="2" t="n">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="L226" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M226" s="2" t="n">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="N226" s="6" t="inlineStr">
         <is>
@@ -13419,13 +13419,13 @@
         <v>396</v>
       </c>
       <c r="K231" s="2" t="n">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="L231" s="2" t="n">
         <v>691</v>
       </c>
       <c r="M231" s="2" t="n">
-        <v>1404</v>
+        <v>1398</v>
       </c>
       <c r="N231" s="4" t="inlineStr">
         <is>
@@ -13704,13 +13704,13 @@
         <v>139</v>
       </c>
       <c r="K236" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="L236" s="2" t="n">
         <v>244</v>
       </c>
       <c r="M236" s="2" t="n">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="N236" s="4" t="inlineStr">
         <is>
@@ -13935,10 +13935,10 @@
         <v>17</v>
       </c>
       <c r="L240" s="2" t="n">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="M240" s="2" t="n">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="N240" s="4" t="inlineStr">
         <is>
@@ -14163,10 +14163,10 @@
         <v>13</v>
       </c>
       <c r="L244" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="M244" s="2" t="n">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N244" s="4" t="inlineStr">
         <is>
@@ -14844,13 +14844,13 @@
         <v>179</v>
       </c>
       <c r="K256" s="2" t="n">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="L256" s="2" t="n">
         <v>129</v>
       </c>
       <c r="M256" s="2" t="n">
-        <v>518</v>
+        <v>510</v>
       </c>
       <c r="N256" s="4" t="inlineStr">
         <is>
@@ -14901,13 +14901,13 @@
         <v>0</v>
       </c>
       <c r="K257" s="2" t="n">
-        <v>283</v>
+        <v>273</v>
       </c>
       <c r="L257" s="2" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="M257" s="2" t="n">
-        <v>412</v>
+        <v>401</v>
       </c>
       <c r="N257" s="6" t="inlineStr">
         <is>
@@ -15075,10 +15075,10 @@
         <v>193</v>
       </c>
       <c r="L260" s="2" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="M260" s="2" t="n">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="N260" s="4" t="inlineStr">
         <is>
@@ -15129,13 +15129,13 @@
         <v>29</v>
       </c>
       <c r="K261" s="2" t="n">
-        <v>151</v>
+        <v>106</v>
       </c>
       <c r="L261" s="2" t="n">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="M261" s="2" t="n">
-        <v>187</v>
+        <v>163</v>
       </c>
       <c r="N261" s="4" t="inlineStr">
         <is>
@@ -15303,10 +15303,10 @@
         <v>46</v>
       </c>
       <c r="L264" s="2" t="n">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="M264" s="2" t="n">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="N264" s="4" t="inlineStr">
         <is>
@@ -15357,13 +15357,13 @@
         <v>29</v>
       </c>
       <c r="K265" s="2" t="n">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="L265" s="2" t="n">
         <v>49</v>
       </c>
       <c r="M265" s="2" t="n">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="N265" s="4" t="inlineStr">
         <is>
@@ -15474,10 +15474,10 @@
         <v>13</v>
       </c>
       <c r="L267" s="2" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="M267" s="2" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N267" s="4" t="inlineStr">
         <is>
@@ -15585,13 +15585,13 @@
         <v>13</v>
       </c>
       <c r="K269" s="2" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="L269" s="2" t="n">
         <v>40</v>
       </c>
       <c r="M269" s="2" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="N269" s="4" t="inlineStr">
         <is>
@@ -15642,13 +15642,13 @@
         <v>55</v>
       </c>
       <c r="K270" s="2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="L270" s="2" t="n">
         <v>74</v>
       </c>
       <c r="M270" s="2" t="n">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="N270" s="4" t="inlineStr">
         <is>
@@ -15870,13 +15870,13 @@
         <v>39</v>
       </c>
       <c r="K274" s="2" t="n">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="L274" s="2" t="n">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="M274" s="2" t="n">
-        <v>381</v>
+        <v>374</v>
       </c>
       <c r="N274" s="4" t="inlineStr">
         <is>
@@ -15930,10 +15930,10 @@
         <v>59</v>
       </c>
       <c r="L275" s="2" t="n">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="M275" s="2" t="n">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="N275" s="4" t="inlineStr">
         <is>
@@ -16836,7 +16836,7 @@
         </is>
       </c>
       <c r="J291" s="2" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="K291" s="2" t="n">
         <v>65</v>
@@ -16845,7 +16845,7 @@
         <v>54</v>
       </c>
       <c r="M291" s="2" t="n">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="N291" s="4" t="inlineStr">
         <is>
@@ -17010,13 +17010,13 @@
         <v>159</v>
       </c>
       <c r="K294" s="2" t="n">
-        <v>342</v>
+        <v>302</v>
       </c>
       <c r="L294" s="2" t="n">
         <v>105</v>
       </c>
       <c r="M294" s="2" t="n">
-        <v>606</v>
+        <v>566</v>
       </c>
       <c r="N294" s="4" t="inlineStr">
         <is>
@@ -17409,13 +17409,13 @@
         <v>50</v>
       </c>
       <c r="K301" s="2" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="L301" s="2" t="n">
         <v>77</v>
       </c>
       <c r="M301" s="2" t="n">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="N301" s="4" t="inlineStr">
         <is>
@@ -17523,13 +17523,13 @@
         <v>26</v>
       </c>
       <c r="K303" s="2" t="n">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="L303" s="2" t="n">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="M303" s="2" t="n">
-        <v>196</v>
+        <v>179</v>
       </c>
       <c r="N303" s="4" t="inlineStr">
         <is>
@@ -17919,7 +17919,7 @@
         </is>
       </c>
       <c r="J310" s="2" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="K310" s="2" t="n">
         <v>54</v>
@@ -17928,7 +17928,7 @@
         <v>6</v>
       </c>
       <c r="M310" s="2" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="N310" s="4" t="inlineStr">
         <is>
@@ -18435,13 +18435,13 @@
         <v>76</v>
       </c>
       <c r="K319" s="2" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="L319" s="2" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="M319" s="2" t="n">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="N319" s="4" t="inlineStr">
         <is>
@@ -19404,10 +19404,10 @@
         <v>22</v>
       </c>
       <c r="K336" s="2" t="n">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="L336" s="2" t="n">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="M336" s="2" t="n">
         <v>116</v>
@@ -19749,10 +19749,10 @@
         <v>92</v>
       </c>
       <c r="L342" s="2" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="M342" s="2" t="n">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="N342" s="4" t="inlineStr">
         <is>
@@ -20145,13 +20145,13 @@
         <v>99</v>
       </c>
       <c r="K349" s="2" t="n">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="L349" s="2" t="n">
         <v>168</v>
       </c>
       <c r="M349" s="2" t="n">
-        <v>521</v>
+        <v>513</v>
       </c>
       <c r="N349" s="4" t="inlineStr">
         <is>
@@ -21057,17 +21057,17 @@
         <v>0</v>
       </c>
       <c r="K365" s="2" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="L365" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M365" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="N365" s="5" t="inlineStr">
-        <is>
-          <t>Sin stock</t>
+        <v>19</v>
+      </c>
+      <c r="N365" s="6" t="inlineStr">
+        <is>
+          <t>7/10 Días</t>
         </is>
       </c>
       <c r="O365" s="2" t="n">
@@ -21570,13 +21570,13 @@
         <v>0</v>
       </c>
       <c r="K374" s="2" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="L374" s="2" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="M374" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="N374" s="6" t="inlineStr">
         <is>
@@ -21966,16 +21966,16 @@
         </is>
       </c>
       <c r="J381" s="2" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="K381" s="2" t="n">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="L381" s="2" t="n">
         <v>94</v>
       </c>
       <c r="M381" s="2" t="n">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="N381" s="4" t="inlineStr">
         <is>
@@ -22254,10 +22254,10 @@
         <v>74</v>
       </c>
       <c r="K386" s="2" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="L386" s="2" t="n">
-        <v>5</v>
+        <v>44</v>
       </c>
       <c r="M386" s="2" t="n">
         <v>118</v>
@@ -22938,13 +22938,13 @@
         <v>0</v>
       </c>
       <c r="K398" s="2" t="n">
-        <v>223</v>
+        <v>194</v>
       </c>
       <c r="L398" s="2" t="n">
         <v>53</v>
       </c>
       <c r="M398" s="2" t="n">
-        <v>276</v>
+        <v>247</v>
       </c>
       <c r="N398" s="6" t="inlineStr">
         <is>
@@ -23047,7 +23047,7 @@
         </is>
       </c>
       <c r="J400" s="2" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K400" s="2" t="n">
         <v>0</v>
@@ -23056,7 +23056,7 @@
         <v>794</v>
       </c>
       <c r="M400" s="2" t="n">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="N400" s="4" t="inlineStr">
         <is>
@@ -23105,13 +23105,13 @@
         <v>0</v>
       </c>
       <c r="K401" s="2" t="n">
-        <v>845</v>
+        <v>825</v>
       </c>
       <c r="L401" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M401" s="2" t="n">
-        <v>845</v>
+        <v>825</v>
       </c>
       <c r="N401" s="6" t="inlineStr">
         <is>
@@ -23270,13 +23270,13 @@
         <v>178</v>
       </c>
       <c r="K404" s="2" t="n">
-        <v>98</v>
+        <v>311</v>
       </c>
       <c r="L404" s="2" t="n">
         <v>54</v>
       </c>
       <c r="M404" s="2" t="n">
-        <v>330</v>
+        <v>543</v>
       </c>
       <c r="N404" s="4" t="inlineStr">
         <is>
@@ -23555,13 +23555,13 @@
         <v>80</v>
       </c>
       <c r="K409" s="2" t="n">
-        <v>560</v>
+        <v>570</v>
       </c>
       <c r="L409" s="2" t="n">
         <v>168</v>
       </c>
       <c r="M409" s="2" t="n">
-        <v>808</v>
+        <v>818</v>
       </c>
       <c r="N409" s="4" t="inlineStr">
         <is>
@@ -23615,10 +23615,10 @@
         <v>682</v>
       </c>
       <c r="L410" s="2" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="M410" s="2" t="n">
-        <v>852</v>
+        <v>850</v>
       </c>
       <c r="N410" s="4" t="inlineStr">
         <is>
@@ -23669,13 +23669,13 @@
         <v>6</v>
       </c>
       <c r="K411" s="2" t="n">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="L411" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M411" s="2" t="n">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="N411" s="6" t="inlineStr">
         <is>
@@ -23897,13 +23897,13 @@
         <v>138</v>
       </c>
       <c r="K415" s="2" t="n">
-        <v>1091</v>
+        <v>1071</v>
       </c>
       <c r="L415" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M415" s="2" t="n">
-        <v>1229</v>
+        <v>1209</v>
       </c>
       <c r="N415" s="4" t="inlineStr">
         <is>
@@ -23954,13 +23954,13 @@
         <v>242</v>
       </c>
       <c r="K416" s="2" t="n">
-        <v>1899</v>
+        <v>1880</v>
       </c>
       <c r="L416" s="2" t="n">
-        <v>655</v>
+        <v>605</v>
       </c>
       <c r="M416" s="2" t="n">
-        <v>2796</v>
+        <v>2727</v>
       </c>
       <c r="N416" s="4" t="inlineStr">
         <is>
@@ -24014,10 +24014,10 @@
         <v>624</v>
       </c>
       <c r="L417" s="2" t="n">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="M417" s="2" t="n">
-        <v>884</v>
+        <v>864</v>
       </c>
       <c r="N417" s="4" t="inlineStr">
         <is>
@@ -24125,13 +24125,13 @@
         <v>279</v>
       </c>
       <c r="K419" s="2" t="n">
-        <v>861</v>
+        <v>580</v>
       </c>
       <c r="L419" s="2" t="n">
-        <v>7</v>
+        <v>237</v>
       </c>
       <c r="M419" s="2" t="n">
-        <v>1147</v>
+        <v>1096</v>
       </c>
       <c r="N419" s="4" t="inlineStr">
         <is>
@@ -24293,16 +24293,16 @@
         </is>
       </c>
       <c r="J422" s="2" t="n">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="K422" s="2" t="n">
-        <v>472</v>
+        <v>450</v>
       </c>
       <c r="L422" s="2" t="n">
         <v>256</v>
       </c>
       <c r="M422" s="2" t="n">
-        <v>830</v>
+        <v>796</v>
       </c>
       <c r="N422" s="4" t="inlineStr">
         <is>
@@ -24752,13 +24752,13 @@
         <v>179</v>
       </c>
       <c r="K430" s="2" t="n">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="L430" s="2" t="n">
         <v>224</v>
       </c>
       <c r="M430" s="2" t="n">
-        <v>543</v>
+        <v>538</v>
       </c>
       <c r="N430" s="4" t="inlineStr">
         <is>
@@ -24923,13 +24923,13 @@
         <v>225</v>
       </c>
       <c r="K433" s="2" t="n">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="L433" s="2" t="n">
         <v>31</v>
       </c>
       <c r="M433" s="2" t="n">
-        <v>453</v>
+        <v>449</v>
       </c>
       <c r="N433" s="4" t="inlineStr">
         <is>
@@ -24983,10 +24983,10 @@
         <v>12</v>
       </c>
       <c r="L434" s="2" t="n">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="M434" s="2" t="n">
-        <v>241</v>
+        <v>217</v>
       </c>
       <c r="N434" s="4" t="inlineStr">
         <is>
@@ -25094,13 +25094,13 @@
         <v>60</v>
       </c>
       <c r="K436" s="2" t="n">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="L436" s="2" t="n">
-        <v>305</v>
+        <v>215</v>
       </c>
       <c r="M436" s="2" t="n">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="N436" s="4" t="inlineStr">
         <is>
@@ -25322,13 +25322,13 @@
         <v>0</v>
       </c>
       <c r="K440" s="2" t="n">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="L440" s="2" t="n">
-        <v>244</v>
+        <v>224</v>
       </c>
       <c r="M440" s="2" t="n">
-        <v>505</v>
+        <v>474</v>
       </c>
       <c r="N440" s="6" t="inlineStr">
         <is>
@@ -25439,10 +25439,10 @@
         <v>219</v>
       </c>
       <c r="L442" s="2" t="n">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="M442" s="2" t="n">
-        <v>709</v>
+        <v>699</v>
       </c>
       <c r="N442" s="4" t="inlineStr">
         <is>
@@ -25550,13 +25550,13 @@
         <v>167</v>
       </c>
       <c r="K444" s="2" t="n">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="L444" s="2" t="n">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="M444" s="2" t="n">
-        <v>502</v>
+        <v>482</v>
       </c>
       <c r="N444" s="4" t="inlineStr">
         <is>
@@ -26120,13 +26120,13 @@
         <v>4</v>
       </c>
       <c r="K454" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L454" s="2" t="n">
         <v>260</v>
       </c>
       <c r="M454" s="2" t="n">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="N454" s="6" t="inlineStr">
         <is>
@@ -26177,13 +26177,13 @@
         <v>26</v>
       </c>
       <c r="K455" s="2" t="n">
-        <v>3</v>
+        <v>58</v>
       </c>
       <c r="L455" s="2" t="n">
         <v>44</v>
       </c>
       <c r="M455" s="2" t="n">
-        <v>73</v>
+        <v>128</v>
       </c>
       <c r="N455" s="4" t="inlineStr">
         <is>
@@ -26234,13 +26234,13 @@
         <v>0</v>
       </c>
       <c r="K456" s="2" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="L456" s="2" t="n">
-        <v>111</v>
+        <v>139</v>
       </c>
       <c r="M456" s="2" t="n">
-        <v>167</v>
+        <v>139</v>
       </c>
       <c r="N456" s="6" t="inlineStr">
         <is>
@@ -26291,13 +26291,13 @@
         <v>352</v>
       </c>
       <c r="K457" s="2" t="n">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="L457" s="2" t="n">
         <v>266</v>
       </c>
       <c r="M457" s="2" t="n">
-        <v>774</v>
+        <v>764</v>
       </c>
       <c r="N457" s="4" t="inlineStr">
         <is>
@@ -26348,13 +26348,13 @@
         <v>275</v>
       </c>
       <c r="K458" s="2" t="n">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="L458" s="2" t="n">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="M458" s="2" t="n">
-        <v>700</v>
+        <v>687</v>
       </c>
       <c r="N458" s="4" t="inlineStr">
         <is>
@@ -26459,20 +26459,20 @@
         </is>
       </c>
       <c r="J460" s="2" t="n">
-        <v>1</v>
+        <v>616</v>
       </c>
       <c r="K460" s="2" t="n">
-        <v>339</v>
+        <v>43</v>
       </c>
       <c r="L460" s="2" t="n">
-        <v>292</v>
+        <v>128</v>
       </c>
       <c r="M460" s="2" t="n">
-        <v>632</v>
-      </c>
-      <c r="N460" s="6" t="inlineStr">
-        <is>
-          <t>7/10 Días</t>
+        <v>787</v>
+      </c>
+      <c r="N460" s="4" t="inlineStr">
+        <is>
+          <t>Stock</t>
         </is>
       </c>
       <c r="O460" s="2" t="n">
@@ -26519,13 +26519,13 @@
         <v>26</v>
       </c>
       <c r="K461" s="2" t="n">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="L461" s="2" t="n">
         <v>24</v>
       </c>
       <c r="M461" s="2" t="n">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="N461" s="4" t="inlineStr">
         <is>
@@ -26576,13 +26576,13 @@
         <v>98</v>
       </c>
       <c r="K462" s="2" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="L462" s="2" t="n">
         <v>85</v>
       </c>
       <c r="M462" s="2" t="n">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="N462" s="4" t="inlineStr">
         <is>
@@ -27032,13 +27032,13 @@
         <v>8</v>
       </c>
       <c r="K470" s="2" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="L470" s="2" t="n">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="M470" s="2" t="n">
-        <v>221</v>
+        <v>208</v>
       </c>
       <c r="N470" s="6" t="inlineStr">
         <is>
@@ -27203,13 +27203,13 @@
         <v>11</v>
       </c>
       <c r="K473" s="2" t="n">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="L473" s="2" t="n">
         <v>91</v>
       </c>
       <c r="M473" s="2" t="n">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="N473" s="4" t="inlineStr">
         <is>
@@ -27257,7 +27257,7 @@
         </is>
       </c>
       <c r="J474" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K474" s="2" t="n">
         <v>138</v>
@@ -27266,7 +27266,7 @@
         <v>81</v>
       </c>
       <c r="M474" s="2" t="n">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="N474" s="4" t="inlineStr">
         <is>
@@ -27488,13 +27488,13 @@
         <v>1</v>
       </c>
       <c r="K478" s="2" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="L478" s="2" t="n">
         <v>3</v>
       </c>
       <c r="M478" s="2" t="n">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="N478" s="6" t="inlineStr">
         <is>

</xml_diff>